<commit_message>
added email field to coach profile along with editField functionality
</commit_message>
<xml_diff>
--- a/public/documentation/Product/MPC Biweekly March 2025.xlsx
+++ b/public/documentation/Product/MPC Biweekly March 2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28803"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omkar\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1719" documentId="8_{7A435C5F-1201-466C-8ED3-86677A3D47AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FAFE06F-EA92-48B5-980E-5B1F5A71BE9B}"/>
+  <xr:revisionPtr revIDLastSave="1909" documentId="8_{7A435C5F-1201-466C-8ED3-86677A3D47AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75C2F0F0-F811-45FA-A8D1-FE951B52B381}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="1" activeTab="1" xr2:uid="{3313DB6C-CF8B-4851-9262-943B759B9BFF}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1580" uniqueCount="385">
   <si>
     <t xml:space="preserve">pin </t>
   </si>
@@ -583,6 +583,15 @@
 2. Also worked on dashbaord making</t>
   </si>
   <si>
+    <t>Completed dashboard making.</t>
+  </si>
+  <si>
+    <t>made some required changes in the dashboard</t>
+  </si>
+  <si>
+    <t>Updated the dashbaord according to the bugs raised in the team.</t>
+  </si>
+  <si>
     <t>Finalized login backend implementation and Completed final login integration.</t>
   </si>
   <si>
@@ -595,12 +604,22 @@
     <t>Fixed bugs and added the character limit to coach profile</t>
   </si>
   <si>
+    <t>1. Added data in tournaments card
+2. Various bugs fixing</t>
+  </si>
+  <si>
     <t>Rendered 2 new fields in tournaments page and tested 50 prompts for MPC Bot</t>
   </si>
   <si>
     <t>Made frontend layout changes in tournment page and performed smoke testing on MPC Bot</t>
   </si>
   <si>
+    <t xml:space="preserve"> Performed smoke testing  for MPC Bot</t>
+  </si>
+  <si>
+    <t>Minor Frontend Changes</t>
+  </si>
+  <si>
     <t>Created Login form</t>
   </si>
   <si>
@@ -620,6 +639,13 @@
   </si>
   <si>
     <t>Changed font size ,style and added scrollbar in tournaments page</t>
+  </si>
+  <si>
+    <t>Implemented bold text issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enhanced UI of Edit tournament,tournament,and dashboard
+</t>
   </si>
   <si>
     <t>WO</t>
@@ -630,6 +656,9 @@
   <si>
     <t>1. Add charcter limit to input field into editTournament Page
 2. Image validation into editTournament Page</t>
+  </si>
+  <si>
+    <t>Two dynamic input field in editTournament</t>
   </si>
   <si>
     <t>Documentation and sent meeting summary to stakeholder</t>
@@ -670,7 +699,7 @@
 2.  Checked in with developers to monitor progress and suggest necessary feedbacks</t>
   </si>
   <si>
-    <t>1. Ask the developers to review the user story and gather relevant feedback.
+    <t>1. Ask the developers to review the user story and provide relevant feedback.
 2. Checked in with developers to monitor progress and suggest necessary feedbacks</t>
   </si>
   <si>
@@ -706,6 +735,24 @@
     <t>1.Solved techincal problems</t>
   </si>
   <si>
+    <t>Fixed bugs</t>
+  </si>
+  <si>
+    <t>Created file directory</t>
+  </si>
+  <si>
+    <t>File directory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fix login page bugs, </t>
+  </si>
+  <si>
+    <t>Resolved edit tournament bugs and updated document files</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
     <t>Fine tuning of Chatbot</t>
   </si>
   <si>
@@ -727,6 +774,9 @@
 2. Added functionality to send one prompt at a time</t>
   </si>
   <si>
+    <t>Added Default Prompts in Chatbot</t>
+  </si>
+  <si>
     <t>Fine tuning of chatbot and worked on Power Bi dashboard</t>
   </si>
   <si>
@@ -788,6 +838,12 @@
   </si>
   <si>
     <t>Added character limit in forms and validations to images</t>
+  </si>
+  <si>
+    <t>Connected Coach Page to Backend and some minor changes</t>
+  </si>
+  <si>
+    <t>Back Button changed and minor issues fixed</t>
   </si>
   <si>
     <t xml:space="preserve">1. Team Members updated data is added
@@ -802,6 +858,9 @@
   </si>
   <si>
     <t>Credit Page background implemented and fix some minor changes</t>
+  </si>
+  <si>
+    <t>Team member score card Scrollbar minor issues fix</t>
   </si>
   <si>
     <t>Name</t>
@@ -1291,7 +1350,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1386,6 +1445,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC0E4F5"/>
         <bgColor rgb="FFC0E4F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1736,11 +1801,32 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="15" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="9" xfId="2" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1753,27 +1839,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2555,10 +2620,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" s="17" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="66" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="21">
@@ -2635,8 +2700,8 @@
       <c r="AL1" s="21"/>
     </row>
     <row r="2" spans="1:38" s="23" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65"/>
+      <c r="A2" s="66"/>
+      <c r="B2" s="66"/>
       <c r="C2" s="21" t="s">
         <v>2</v>
       </c>
@@ -4435,7 +4500,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C175BB12-9F93-43B1-9AA8-D08E8CD4B089}">
-  <dimension ref="A1:BH28"/>
+  <dimension ref="A1:BJ28"/>
   <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="4" customWidth="1"/>
@@ -4484,138 +4549,144 @@
     <col min="44" max="44" width="12.85546875" style="1" customWidth="1"/>
     <col min="45" max="50" width="20.7109375" style="1"/>
     <col min="51" max="51" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="52" max="16372" width="20.7109375" style="1"/>
+    <col min="52" max="58" width="20.7109375" style="1"/>
+    <col min="59" max="59" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="60" max="16372" width="20.7109375" style="1"/>
     <col min="16373" max="16376" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="16377" max="16384" width="20.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" s="17" customFormat="1">
-      <c r="A1" s="65" t="s">
+    <row r="1" spans="1:62" s="17" customFormat="1">
+      <c r="A1" s="66" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="66">
+      <c r="C1" s="67">
         <v>45727</v>
       </c>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66">
+      <c r="D1" s="67"/>
+      <c r="E1" s="67">
         <v>45728</v>
       </c>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66">
+      <c r="F1" s="67"/>
+      <c r="G1" s="67">
         <v>45729</v>
       </c>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66">
+      <c r="H1" s="67"/>
+      <c r="I1" s="67">
         <v>45730</v>
       </c>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66">
+      <c r="J1" s="67"/>
+      <c r="K1" s="67">
         <v>45731</v>
       </c>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66">
+      <c r="L1" s="67"/>
+      <c r="M1" s="67">
         <v>45732</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66">
+      <c r="N1" s="67"/>
+      <c r="O1" s="67">
         <v>45733</v>
       </c>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66">
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67">
         <v>45734</v>
       </c>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66">
+      <c r="R1" s="67"/>
+      <c r="S1" s="67">
         <v>45735</v>
       </c>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66">
+      <c r="T1" s="67"/>
+      <c r="U1" s="67">
         <v>45736</v>
       </c>
-      <c r="V1" s="66"/>
-      <c r="W1" s="66">
+      <c r="V1" s="67"/>
+      <c r="W1" s="67">
         <v>45737</v>
       </c>
-      <c r="X1" s="66"/>
-      <c r="Y1" s="66">
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67">
         <v>45738</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66">
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67">
         <v>45739</v>
       </c>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66">
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67">
         <v>45740</v>
       </c>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66">
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67">
         <v>45741</v>
       </c>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66">
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67">
         <v>45742</v>
       </c>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="66">
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67">
         <v>45743</v>
       </c>
-      <c r="AJ1" s="66"/>
-      <c r="AK1" s="66">
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67">
         <v>45744</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66">
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67">
         <v>45745</v>
       </c>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66">
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67">
         <v>45746</v>
       </c>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66">
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67">
         <v>45747</v>
       </c>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66">
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67">
         <v>45748</v>
       </c>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="66">
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67">
         <v>45749</v>
       </c>
-      <c r="AV1" s="66"/>
-      <c r="AW1" s="66">
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="67">
         <v>45750</v>
       </c>
-      <c r="AX1" s="66"/>
-      <c r="AY1" s="66">
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67">
         <v>45751</v>
       </c>
-      <c r="AZ1" s="66"/>
-      <c r="BA1" s="66">
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="67">
         <v>45752</v>
       </c>
-      <c r="BB1" s="66"/>
-      <c r="BC1" s="66">
+      <c r="BB1" s="67"/>
+      <c r="BC1" s="67">
         <v>45753</v>
       </c>
-      <c r="BD1" s="66"/>
-      <c r="BE1" s="66">
+      <c r="BD1" s="67"/>
+      <c r="BE1" s="67">
         <v>45754</v>
       </c>
-      <c r="BF1" s="66"/>
-      <c r="BG1" s="66">
+      <c r="BF1" s="67"/>
+      <c r="BG1" s="67">
         <v>45755</v>
       </c>
-      <c r="BH1" s="66"/>
-    </row>
-    <row r="2" spans="1:60" s="17" customFormat="1">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65"/>
+      <c r="BH1" s="67"/>
+      <c r="BI1" s="67">
+        <v>45756</v>
+      </c>
+      <c r="BJ1" s="67"/>
+    </row>
+    <row r="2" spans="1:62" s="17" customFormat="1">
+      <c r="A2" s="66"/>
+      <c r="B2" s="66"/>
       <c r="C2" s="42" t="s">
         <v>2</v>
       </c>
@@ -4790,8 +4861,14 @@
       <c r="BH2" s="43" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:60" ht="121.5">
+      <c r="BI2" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="BJ2" s="43" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:62" ht="121.5">
       <c r="A3" s="44">
         <v>1</v>
       </c>
@@ -4910,24 +4987,44 @@
       <c r="AR3" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="AS3" s="44"/>
+      <c r="AS3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AT3" s="44"/>
-      <c r="AU3" s="44"/>
+      <c r="AU3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AV3" s="44"/>
-      <c r="AW3" s="44"/>
+      <c r="AW3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AX3" s="44"/>
-      <c r="AY3" s="44"/>
+      <c r="AY3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ3" s="44"/>
-      <c r="BA3" s="44"/>
+      <c r="BA3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB3" s="44"/>
-      <c r="BC3" s="44"/>
+      <c r="BC3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD3" s="44"/>
-      <c r="BE3" s="44"/>
+      <c r="BE3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF3" s="44"/>
-      <c r="BG3" s="44"/>
+      <c r="BG3" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BH3" s="44"/>
-    </row>
-    <row r="4" spans="1:60" ht="137.25">
+      <c r="BI3" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ3" s="44"/>
+    </row>
+    <row r="4" spans="1:62" ht="137.25">
       <c r="A4" s="45">
         <v>2</v>
       </c>
@@ -5046,24 +5143,50 @@
       <c r="AR4" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="AS4" s="45"/>
-      <c r="AT4" s="45"/>
-      <c r="AU4" s="45"/>
-      <c r="AV4" s="45"/>
-      <c r="AW4" s="45"/>
+      <c r="AS4" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT4" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="AU4" s="45" t="s">
+        <v>168</v>
+      </c>
+      <c r="AV4" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="AW4" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="AX4" s="45"/>
-      <c r="AY4" s="45"/>
-      <c r="AZ4" s="45"/>
-      <c r="BA4" s="45"/>
+      <c r="AY4" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="AZ4" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="BA4" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BB4" s="45"/>
-      <c r="BC4" s="45"/>
+      <c r="BC4" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BD4" s="45"/>
-      <c r="BE4" s="45"/>
+      <c r="BE4" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BF4" s="45"/>
-      <c r="BG4" s="45"/>
+      <c r="BG4" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BH4" s="45"/>
-    </row>
-    <row r="5" spans="1:60" ht="76.5">
+      <c r="BI4" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ4" s="45"/>
+    </row>
+    <row r="5" spans="1:62" ht="76.5">
       <c r="A5" s="44">
         <v>3</v>
       </c>
@@ -5137,7 +5260,7 @@
         <v>19</v>
       </c>
       <c r="AE5" s="44" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AF5" s="44" t="s">
         <v>10</v>
@@ -5169,13 +5292,13 @@
       </c>
       <c r="AP5" s="44"/>
       <c r="AQ5" s="44" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="AR5" s="50" t="s">
         <v>10</v>
       </c>
       <c r="AS5" s="44" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AT5" s="44" t="s">
         <v>10</v>
@@ -5185,23 +5308,39 @@
       </c>
       <c r="AV5" s="44"/>
       <c r="AW5" s="44" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AX5" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="AY5" s="44"/>
+      <c r="AY5" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ5" s="44"/>
-      <c r="BA5" s="44"/>
+      <c r="BA5" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB5" s="44"/>
-      <c r="BC5" s="44"/>
+      <c r="BC5" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD5" s="44"/>
-      <c r="BE5" s="44"/>
+      <c r="BE5" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF5" s="44"/>
-      <c r="BG5" s="44"/>
-      <c r="BH5" s="44"/>
-    </row>
-    <row r="6" spans="1:60" ht="76.5">
+      <c r="BG5" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="BH5" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI5" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ5" s="44"/>
+    </row>
+    <row r="6" spans="1:62" ht="76.5">
       <c r="A6" s="45">
         <v>4</v>
       </c>
@@ -5307,29 +5446,33 @@
       </c>
       <c r="AP6" s="45"/>
       <c r="AQ6" s="45" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="AR6" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS6" s="45" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="AT6" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="AU6" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="AV6" s="45"/>
+      <c r="AU6" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="AV6" s="45" t="s">
+        <v>17</v>
+      </c>
       <c r="AW6" s="45" t="s">
         <v>5</v>
       </c>
       <c r="AX6" s="45"/>
       <c r="AY6" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="AZ6" s="45"/>
+        <v>178</v>
+      </c>
+      <c r="AZ6" s="45" t="s">
+        <v>17</v>
+      </c>
       <c r="BA6" s="45" t="s">
         <v>5</v>
       </c>
@@ -5342,10 +5485,16 @@
         <v>5</v>
       </c>
       <c r="BF6" s="45"/>
-      <c r="BG6" s="45"/>
+      <c r="BG6" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BH6" s="45"/>
-    </row>
-    <row r="7" spans="1:60" ht="60.75">
+      <c r="BI6" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ6" s="45"/>
+    </row>
+    <row r="7" spans="1:62" ht="60.75">
       <c r="A7" s="44">
         <v>5</v>
       </c>
@@ -5445,25 +5594,25 @@
       </c>
       <c r="AN7" s="44"/>
       <c r="AO7" s="44" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="AP7" s="44" t="s">
         <v>33</v>
       </c>
       <c r="AQ7" s="44" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="AR7" s="50" t="s">
         <v>19</v>
       </c>
       <c r="AS7" s="44" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="AT7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AU7" s="44" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="AV7" s="44" t="s">
         <v>10</v>
@@ -5492,8 +5641,12 @@
         <v>5</v>
       </c>
       <c r="BH7" s="44"/>
-    </row>
-    <row r="8" spans="1:60" ht="76.5">
+      <c r="BI7" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ7" s="44"/>
+    </row>
+    <row r="8" spans="1:62" ht="76.5">
       <c r="A8" s="45">
         <v>6</v>
       </c>
@@ -5599,13 +5752,13 @@
       </c>
       <c r="AP8" s="45"/>
       <c r="AQ8" s="45" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="AR8" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS8" s="45" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="AT8" s="45" t="s">
         <v>10</v>
@@ -5615,23 +5768,41 @@
       </c>
       <c r="AV8" s="45"/>
       <c r="AW8" s="45" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AX8" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="AY8" s="45"/>
+      <c r="AY8" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ8" s="45"/>
-      <c r="BA8" s="45"/>
+      <c r="BA8" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BB8" s="45"/>
-      <c r="BC8" s="45"/>
+      <c r="BC8" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BD8" s="45"/>
-      <c r="BE8" s="45"/>
+      <c r="BE8" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BF8" s="45"/>
-      <c r="BG8" s="45"/>
-      <c r="BH8" s="45"/>
-    </row>
-    <row r="9" spans="1:60" ht="91.5">
+      <c r="BG8" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="BH8" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI8" s="45" t="s">
+        <v>187</v>
+      </c>
+      <c r="BJ8" s="45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:62" ht="91.5">
       <c r="A9" s="44">
         <v>7</v>
       </c>
@@ -5740,13 +5911,13 @@
         <v>5</v>
       </c>
       <c r="AN9" s="44" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AO9" s="44" t="s">
         <v>5</v>
       </c>
       <c r="AP9" s="44" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AQ9" s="44" t="s">
         <v>5</v>
@@ -5755,7 +5926,7 @@
         <v>47</v>
       </c>
       <c r="AS9" s="44" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="AT9" s="44" t="s">
         <v>10</v>
@@ -5765,23 +5936,39 @@
       </c>
       <c r="AV9" s="44"/>
       <c r="AW9" s="44" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="AX9" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="AY9" s="44"/>
+      <c r="AY9" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ9" s="44"/>
-      <c r="BA9" s="44"/>
+      <c r="BA9" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB9" s="44"/>
-      <c r="BC9" s="44"/>
+      <c r="BC9" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD9" s="44"/>
-      <c r="BE9" s="44"/>
+      <c r="BE9" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF9" s="44"/>
-      <c r="BG9" s="44"/>
-      <c r="BH9" s="44"/>
-    </row>
-    <row r="10" spans="1:60" ht="183">
+      <c r="BG9" s="44" t="s">
+        <v>191</v>
+      </c>
+      <c r="BH9" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI9" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ9" s="44"/>
+    </row>
+    <row r="10" spans="1:62" ht="183">
       <c r="A10" s="45">
         <v>8</v>
       </c>
@@ -5810,13 +5997,13 @@
         <v>5</v>
       </c>
       <c r="J10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="K10" s="45" t="s">
         <v>5</v>
       </c>
       <c r="L10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="M10" s="45" t="s">
         <v>89</v>
@@ -5858,13 +6045,13 @@
         <v>5</v>
       </c>
       <c r="Z10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AA10" s="45" t="s">
         <v>5</v>
       </c>
       <c r="AB10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AC10" s="45" t="s">
         <v>95</v>
@@ -5891,7 +6078,7 @@
         <v>10</v>
       </c>
       <c r="AK10" s="45" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="AL10" s="45" t="s">
         <v>10</v>
@@ -5900,46 +6087,66 @@
         <v>5</v>
       </c>
       <c r="AN10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AO10" s="45" t="s">
         <v>5</v>
       </c>
       <c r="AP10" s="45" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="AQ10" s="45" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AR10" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS10" s="45" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="AT10" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AU10" s="45" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AV10" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="AW10" s="45"/>
-      <c r="AX10" s="45"/>
-      <c r="AY10" s="45"/>
-      <c r="AZ10" s="45"/>
-      <c r="BA10" s="45"/>
+      <c r="AW10" s="45" t="s">
+        <v>193</v>
+      </c>
+      <c r="AX10" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY10" s="45" t="s">
+        <v>193</v>
+      </c>
+      <c r="AZ10" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="BA10" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB10" s="45"/>
-      <c r="BC10" s="45"/>
+      <c r="BC10" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD10" s="45"/>
-      <c r="BE10" s="45"/>
+      <c r="BE10" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BF10" s="45"/>
-      <c r="BG10" s="45"/>
+      <c r="BG10" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BH10" s="45"/>
-    </row>
-    <row r="11" spans="1:60" ht="121.5">
+      <c r="BI10" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ10" s="45"/>
+    </row>
+    <row r="11" spans="1:62" ht="121.5">
       <c r="A11" s="44">
         <v>9</v>
       </c>
@@ -5947,7 +6154,7 @@
         <v>100</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="D11" s="44" t="s">
         <v>10</v>
@@ -5995,13 +6202,13 @@
         <v>5</v>
       </c>
       <c r="S11" s="44" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="T11" s="44" t="s">
         <v>10</v>
       </c>
       <c r="U11" s="44" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="V11" s="44" t="s">
         <v>10</v>
@@ -6015,23 +6222,17 @@
       <c r="Y11" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="Z11" s="44" t="s">
-        <v>5</v>
-      </c>
+      <c r="Z11" s="44"/>
       <c r="AA11" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="AB11" s="44" t="s">
-        <v>5</v>
-      </c>
+      <c r="AB11" s="44"/>
       <c r="AC11" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="AD11" s="44" t="s">
-        <v>5</v>
-      </c>
+      <c r="AD11" s="44"/>
       <c r="AE11" s="44" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="AF11" s="44" t="s">
         <v>10</v>
@@ -6049,7 +6250,7 @@
         <v>10</v>
       </c>
       <c r="AK11" s="44" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="AL11" s="44" t="s">
         <v>10</v>
@@ -6063,51 +6264,57 @@
       </c>
       <c r="AP11" s="44"/>
       <c r="AQ11" s="44" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="AR11" s="50" t="s">
         <v>10</v>
       </c>
       <c r="AS11" s="44" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="AT11" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AU11" s="44" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="AV11" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AW11" s="44" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="AX11" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="AY11" s="77" t="s">
-        <v>193</v>
+      <c r="AY11" s="65" t="s">
+        <v>202</v>
       </c>
       <c r="AZ11" s="44" t="s">
-        <v>17</v>
-      </c>
-      <c r="BA11" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="BA11" s="44" t="s">
         <v>5</v>
       </c>
       <c r="BB11" s="44"/>
-      <c r="BC11" s="22" t="s">
+      <c r="BC11" s="44" t="s">
         <v>5</v>
       </c>
       <c r="BD11" s="44"/>
-      <c r="BE11" s="22" t="s">
+      <c r="BE11" s="44" t="s">
         <v>5</v>
       </c>
       <c r="BF11" s="44"/>
-      <c r="BG11" s="44"/>
+      <c r="BG11" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BH11" s="44"/>
-    </row>
-    <row r="12" spans="1:60" ht="183">
+      <c r="BI11" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ11" s="44"/>
+    </row>
+    <row r="12" spans="1:62" ht="183">
       <c r="A12" s="45">
         <v>10</v>
       </c>
@@ -6157,7 +6364,7 @@
         <v>47</v>
       </c>
       <c r="Q12" s="45" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="R12" s="45" t="s">
         <v>10</v>
@@ -6219,13 +6426,13 @@
       </c>
       <c r="AP12" s="45"/>
       <c r="AQ12" s="45" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="AR12" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS12" s="45" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="AT12" s="45" t="s">
         <v>10</v>
@@ -6258,10 +6465,16 @@
       <c r="BF12" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="BG12" s="45"/>
+      <c r="BG12" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BH12" s="45"/>
-    </row>
-    <row r="13" spans="1:60" ht="76.5">
+      <c r="BI12" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ12" s="45"/>
+    </row>
+    <row r="13" spans="1:62" ht="76.5">
       <c r="A13" s="44">
         <v>11</v>
       </c>
@@ -6365,13 +6578,13 @@
         <v>10</v>
       </c>
       <c r="AI13" s="44" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="AJ13" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AK13" s="44" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="AL13" s="44" t="s">
         <v>19</v>
@@ -6379,43 +6592,71 @@
       <c r="AM13" s="44"/>
       <c r="AN13" s="44"/>
       <c r="AO13" s="44" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="AP13" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AQ13" s="44" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="AR13" s="50" t="s">
         <v>10</v>
       </c>
       <c r="AS13" s="44" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="AT13" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AU13" s="44" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="AV13" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="AW13" s="44"/>
-      <c r="AX13" s="44"/>
-      <c r="AY13" s="44"/>
-      <c r="AZ13" s="44"/>
-      <c r="BA13" s="44"/>
+      <c r="AW13" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="AX13" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="AY13" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="AZ13" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BA13" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB13" s="44"/>
-      <c r="BC13" s="44"/>
-      <c r="BD13" s="44"/>
-      <c r="BE13" s="44"/>
-      <c r="BF13" s="44"/>
-      <c r="BG13" s="44"/>
-      <c r="BH13" s="44"/>
-    </row>
-    <row r="14" spans="1:60" ht="106.5">
+      <c r="BC13" s="44" t="s">
+        <v>213</v>
+      </c>
+      <c r="BD13" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="BE13" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="BF13" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BG13" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="BH13" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI13" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="BJ13" s="44" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="14" spans="1:62" ht="106.5">
       <c r="A14" s="45">
         <v>12</v>
       </c>
@@ -6539,31 +6780,31 @@
       </c>
       <c r="AP14" s="45"/>
       <c r="AQ14" s="45" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AR14" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS14" s="45" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="AT14" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AU14" s="45" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="AV14" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AW14" s="45" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="AX14" s="45" t="s">
         <v>133</v>
       </c>
       <c r="AY14" s="45" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="AZ14" s="45" t="s">
         <v>10</v>
@@ -6579,15 +6820,21 @@
       <c r="BE14" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="BF14" s="45"/>
+      <c r="BF14" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BG14" s="45" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="BH14" s="45" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:60" ht="76.5">
+      <c r="BI14" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ14" s="45"/>
+    </row>
+    <row r="15" spans="1:62" ht="76.5">
       <c r="A15" s="44">
         <v>13</v>
       </c>
@@ -6681,7 +6928,7 @@
         <v>10</v>
       </c>
       <c r="AK15" s="44" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AL15" s="44" t="s">
         <v>19</v>
@@ -6695,19 +6942,19 @@
       </c>
       <c r="AP15" s="44"/>
       <c r="AQ15" s="44" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AR15" s="50" t="s">
         <v>10</v>
       </c>
       <c r="AS15" s="44" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="AT15" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AU15" s="44" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AV15" s="44" t="s">
         <v>10</v>
@@ -6716,18 +6963,34 @@
         <v>5</v>
       </c>
       <c r="AX15" s="44"/>
-      <c r="AY15" s="44"/>
+      <c r="AY15" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ15" s="44"/>
-      <c r="BA15" s="44"/>
+      <c r="BA15" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB15" s="44"/>
-      <c r="BC15" s="44"/>
+      <c r="BC15" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD15" s="44"/>
-      <c r="BE15" s="44"/>
+      <c r="BE15" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF15" s="44"/>
-      <c r="BG15" s="44"/>
-      <c r="BH15" s="44"/>
-    </row>
-    <row r="16" spans="1:60" ht="45.75">
+      <c r="BG15" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="BH15" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI15" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ15" s="44"/>
+    </row>
+    <row r="16" spans="1:62" ht="45.75">
       <c r="A16" s="45">
         <v>14</v>
       </c>
@@ -6821,7 +7084,7 @@
         <v>10</v>
       </c>
       <c r="AK16" s="45" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AL16" s="45" t="s">
         <v>19</v>
@@ -6831,31 +7094,31 @@
       <c r="AO16" s="45"/>
       <c r="AP16" s="45"/>
       <c r="AQ16" s="45" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AR16" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS16" s="45" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="AT16" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AU16" s="45" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="AV16" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AW16" s="45" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="AX16" s="45" t="s">
         <v>133</v>
       </c>
       <c r="AY16" s="45" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="AZ16" s="45" t="s">
         <v>10</v>
@@ -6873,13 +7136,17 @@
       </c>
       <c r="BF16" s="45"/>
       <c r="BG16" s="45" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="BH16" s="45" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:60" ht="76.5">
+      <c r="BI16" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ16" s="45"/>
+    </row>
+    <row r="17" spans="1:62" ht="76.5">
       <c r="A17" s="44">
         <v>15</v>
       </c>
@@ -6887,25 +7154,25 @@
         <v>144</v>
       </c>
       <c r="C17" s="44" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="F17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="44" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="H17" s="44" t="s">
         <v>73</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="J17" s="44" t="s">
         <v>10</v>
@@ -6919,31 +7186,31 @@
       </c>
       <c r="N17" s="44"/>
       <c r="O17" s="44" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="P17" s="44" t="s">
         <v>19</v>
       </c>
       <c r="Q17" s="44" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="R17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="S17" s="44" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="T17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="U17" s="44" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="V17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="W17" s="44" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="X17" s="44" t="s">
         <v>10</v>
@@ -6957,83 +7224,101 @@
       </c>
       <c r="AB17" s="44"/>
       <c r="AC17" s="44" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="AD17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AE17" s="44" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="AF17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AG17" s="44" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="AH17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AI17" s="44" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="AJ17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AK17" s="44" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="AL17" s="44" t="s">
         <v>19</v>
       </c>
       <c r="AM17" s="44" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="AN17" s="44" t="s">
         <v>19</v>
       </c>
       <c r="AO17" s="44" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="AP17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AQ17" s="44" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="AR17" s="50" t="s">
         <v>10</v>
       </c>
       <c r="AS17" s="44" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="AT17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AU17" s="44" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="AV17" s="44" t="s">
         <v>10</v>
       </c>
       <c r="AW17" s="44" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="AX17" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="AY17" s="44"/>
-      <c r="AZ17" s="44"/>
-      <c r="BA17" s="44"/>
+      <c r="AY17" s="44" t="s">
+        <v>246</v>
+      </c>
+      <c r="AZ17" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BA17" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB17" s="44"/>
-      <c r="BC17" s="44"/>
+      <c r="BC17" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD17" s="44"/>
-      <c r="BE17" s="44"/>
+      <c r="BE17" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF17" s="44"/>
-      <c r="BG17" s="44"/>
-      <c r="BH17" s="44"/>
-    </row>
-    <row r="18" spans="1:60" ht="91.5">
+      <c r="BG17" s="44" t="s">
+        <v>247</v>
+      </c>
+      <c r="BH17" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI17" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ17" s="44"/>
+    </row>
+    <row r="18" spans="1:62" ht="91.5">
       <c r="A18" s="45">
         <v>16</v>
       </c>
@@ -7153,41 +7438,57 @@
       </c>
       <c r="AP18" s="45"/>
       <c r="AQ18" s="45" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="AR18" s="51" t="s">
         <v>10</v>
       </c>
       <c r="AS18" s="45" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="AT18" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AU18" s="45" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="AV18" s="45" t="s">
         <v>10</v>
       </c>
       <c r="AW18" s="45" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="AX18" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="AY18" s="45"/>
+      <c r="AY18" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ18" s="45"/>
-      <c r="BA18" s="45"/>
+      <c r="BA18" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BB18" s="45"/>
-      <c r="BC18" s="45"/>
+      <c r="BC18" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BD18" s="45"/>
-      <c r="BE18" s="45"/>
+      <c r="BE18" s="45" t="s">
+        <v>5</v>
+      </c>
       <c r="BF18" s="45"/>
-      <c r="BG18" s="45"/>
-      <c r="BH18" s="45"/>
-    </row>
-    <row r="19" spans="1:60" ht="91.5">
+      <c r="BG18" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="BH18" s="45" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI18" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ18" s="45"/>
+    </row>
+    <row r="19" spans="1:62" ht="91.5">
       <c r="A19" s="44">
         <v>17</v>
       </c>
@@ -7296,58 +7597,56 @@
         <v>5</v>
       </c>
       <c r="AX19" s="44"/>
-      <c r="AY19" s="44"/>
+      <c r="AY19" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="AZ19" s="44"/>
-      <c r="BA19" s="44"/>
+      <c r="BA19" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BB19" s="44"/>
-      <c r="BC19" s="44"/>
+      <c r="BC19" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BD19" s="44"/>
-      <c r="BE19" s="44"/>
+      <c r="BE19" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BF19" s="44"/>
-      <c r="BG19" s="44"/>
+      <c r="BG19" s="44" t="s">
+        <v>5</v>
+      </c>
       <c r="BH19" s="44"/>
-    </row>
-    <row r="20" spans="1:60">
+      <c r="BI19" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="BJ19" s="44"/>
+    </row>
+    <row r="20" spans="1:62">
       <c r="A20" s="3"/>
     </row>
-    <row r="21" spans="1:60">
+    <row r="21" spans="1:62">
       <c r="A21" s="3"/>
     </row>
-    <row r="22" spans="1:60">
+    <row r="22" spans="1:62">
       <c r="A22" s="3"/>
     </row>
-    <row r="23" spans="1:60">
+    <row r="23" spans="1:62">
       <c r="A23" s="3"/>
     </row>
-    <row r="24" spans="1:60">
+    <row r="24" spans="1:62">
       <c r="A24" s="3"/>
     </row>
-    <row r="25" spans="1:60">
+    <row r="25" spans="1:62">
       <c r="A25" s="5"/>
       <c r="B25" s="2"/>
     </row>
-    <row r="28" spans="1:60">
+    <row r="28" spans="1:62">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="AY1:AZ1"/>
-    <mergeCell ref="BA1:BB1"/>
-    <mergeCell ref="BC1:BD1"/>
-    <mergeCell ref="BE1:BF1"/>
-    <mergeCell ref="BG1:BH1"/>
-    <mergeCell ref="AU1:AV1"/>
-    <mergeCell ref="AW1:AX1"/>
-    <mergeCell ref="AM1:AN1"/>
-    <mergeCell ref="AO1:AP1"/>
-    <mergeCell ref="AQ1:AR1"/>
-    <mergeCell ref="AC1:AD1"/>
-    <mergeCell ref="AE1:AF1"/>
-    <mergeCell ref="AG1:AH1"/>
-    <mergeCell ref="AI1:AJ1"/>
-    <mergeCell ref="AS1:AT1"/>
-    <mergeCell ref="AK1:AL1"/>
+  <mergeCells count="32">
     <mergeCell ref="AA1:AB1"/>
     <mergeCell ref="Y1:Z1"/>
     <mergeCell ref="A1:A2"/>
@@ -7363,6 +7662,23 @@
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="S1:T1"/>
     <mergeCell ref="U1:V1"/>
+    <mergeCell ref="AC1:AD1"/>
+    <mergeCell ref="AE1:AF1"/>
+    <mergeCell ref="AG1:AH1"/>
+    <mergeCell ref="AI1:AJ1"/>
+    <mergeCell ref="AS1:AT1"/>
+    <mergeCell ref="AK1:AL1"/>
+    <mergeCell ref="AU1:AV1"/>
+    <mergeCell ref="AW1:AX1"/>
+    <mergeCell ref="AM1:AN1"/>
+    <mergeCell ref="AO1:AP1"/>
+    <mergeCell ref="AQ1:AR1"/>
+    <mergeCell ref="BI1:BJ1"/>
+    <mergeCell ref="AY1:AZ1"/>
+    <mergeCell ref="BA1:BB1"/>
+    <mergeCell ref="BC1:BD1"/>
+    <mergeCell ref="BE1:BF1"/>
+    <mergeCell ref="BG1:BH1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -7382,27 +7698,27 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="58" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="B1" s="59" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
       <c r="C1" s="59" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="D1" s="60" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="29.25">
       <c r="A2" s="53" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="B2" s="49" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
       <c r="D2" s="55" t="s">
         <v>4</v>
@@ -7410,13 +7726,13 @@
     </row>
     <row r="3" spans="1:4" ht="29.25">
       <c r="A3" s="53" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="D3" s="55" t="s">
         <v>22</v>
@@ -7424,13 +7740,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="52" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>245</v>
+        <v>264</v>
       </c>
       <c r="C4" s="46" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="D4" s="54" t="s">
         <v>31</v>
@@ -7438,27 +7754,27 @@
     </row>
     <row r="5" spans="1:4" ht="29.25">
       <c r="A5" s="52" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="B5" s="47" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>249</v>
+        <v>268</v>
       </c>
       <c r="D5" s="54" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="29.25">
       <c r="A6" s="52" t="s">
-        <v>250</v>
+        <v>269</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>252</v>
+        <v>271</v>
       </c>
       <c r="D6" s="54" t="s">
         <v>51</v>
@@ -7466,55 +7782,55 @@
     </row>
     <row r="7" spans="1:4" ht="29.25">
       <c r="A7" s="53" t="s">
-        <v>253</v>
+        <v>272</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="C7" s="48" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="D7" s="55" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="29.25">
       <c r="A8" s="53" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
       <c r="C8" s="48" t="s">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="D8" s="56" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="87">
       <c r="A9" s="52" t="s">
-        <v>261</v>
+        <v>280</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>262</v>
+        <v>281</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>263</v>
+        <v>282</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="29.25">
       <c r="A10" s="53" t="s">
-        <v>265</v>
+        <v>284</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>266</v>
+        <v>285</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
       <c r="D10" s="55" t="s">
         <v>100</v>
@@ -7522,24 +7838,24 @@
     </row>
     <row r="11" spans="1:4" ht="43.5">
       <c r="A11" s="53" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="B11" s="48" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="D11" s="55" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29.25">
       <c r="A12" s="53" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="C12" s="48" t="s">
         <v>5</v>
@@ -7550,13 +7866,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="52" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B13" s="46" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="D13" s="57" t="s">
         <v>111</v>
@@ -7564,27 +7880,27 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="52" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
       <c r="B14" s="46" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="D14" s="54" t="s">
-        <v>260</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="57.75">
       <c r="A15" s="52" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="B15" s="46" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="C15" s="47" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="D15" s="54" t="s">
         <v>131</v>
@@ -7592,27 +7908,27 @@
     </row>
     <row r="16" spans="1:4" ht="43.5">
       <c r="A16" s="52" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="B16" s="47" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
       <c r="D16" s="54" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="43.5">
       <c r="A17" s="53" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="D17" s="64" t="s">
         <v>144</v>
@@ -7620,13 +7936,13 @@
     </row>
     <row r="18" spans="1:4" ht="29.25">
       <c r="A18" s="53" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="D18" s="56" t="s">
         <v>145</v>
@@ -7634,13 +7950,13 @@
     </row>
     <row r="19" spans="1:4" ht="43.5">
       <c r="A19" s="61" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="B19" s="62" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="C19" s="62" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="D19" s="63" t="s">
         <v>159</v>
@@ -7689,84 +8005,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="76" t="s">
-        <v>296</v>
-      </c>
-      <c r="B1" s="76" t="s">
-        <v>297</v>
-      </c>
-      <c r="C1" s="76" t="s">
-        <v>298</v>
-      </c>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76" t="s">
-        <v>299</v>
-      </c>
-      <c r="F1" s="76"/>
+      <c r="A1" s="68" t="s">
+        <v>315</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>316</v>
+      </c>
+      <c r="C1" s="68" t="s">
+        <v>317</v>
+      </c>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68" t="s">
+        <v>318</v>
+      </c>
+      <c r="F1" s="68"/>
     </row>
     <row r="2" spans="1:7" ht="15">
-      <c r="A2" s="76"/>
-      <c r="B2" s="76"/>
+      <c r="A2" s="68"/>
+      <c r="B2" s="68"/>
       <c r="C2" s="30" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="G2"/>
     </row>
     <row r="3" spans="1:7" ht="15">
-      <c r="A3" s="73">
+      <c r="A3" s="70">
         <v>1</v>
       </c>
-      <c r="B3" s="71" t="s">
-        <v>302</v>
+      <c r="B3" s="69" t="s">
+        <v>321</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>303</v>
-      </c>
-      <c r="D3" s="73" t="s">
-        <v>304</v>
+        <v>322</v>
+      </c>
+      <c r="D3" s="70" t="s">
+        <v>323</v>
       </c>
       <c r="E3" s="32"/>
       <c r="F3" s="32"/>
       <c r="G3"/>
     </row>
     <row r="4" spans="1:7" ht="15">
-      <c r="A4" s="73"/>
-      <c r="B4" s="71"/>
+      <c r="A4" s="70"/>
+      <c r="B4" s="69"/>
       <c r="C4" s="33" t="s">
-        <v>305</v>
-      </c>
-      <c r="D4" s="73"/>
+        <v>324</v>
+      </c>
+      <c r="D4" s="70"/>
       <c r="E4" s="33"/>
       <c r="F4" s="33"/>
       <c r="G4"/>
     </row>
     <row r="5" spans="1:7" ht="15">
-      <c r="A5" s="73"/>
-      <c r="B5" s="71"/>
+      <c r="A5" s="70"/>
+      <c r="B5" s="69"/>
       <c r="C5" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="D5" s="73"/>
+        <v>325</v>
+      </c>
+      <c r="D5" s="70"/>
       <c r="E5" s="32"/>
       <c r="F5" s="32"/>
       <c r="G5"/>
     </row>
     <row r="6" spans="1:7" ht="30.75">
-      <c r="A6" s="73"/>
-      <c r="B6" s="71"/>
+      <c r="A6" s="70"/>
+      <c r="B6" s="69"/>
       <c r="C6" s="33" t="s">
-        <v>307</v>
-      </c>
-      <c r="D6" s="73"/>
+        <v>326</v>
+      </c>
+      <c r="D6" s="70"/>
       <c r="E6" s="33"/>
       <c r="F6" s="33"/>
       <c r="G6"/>
@@ -7776,16 +8092,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D7" s="36" t="s">
         <v>51</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="F7" s="36" t="s">
         <v>31</v>
@@ -7793,128 +8109,128 @@
       <c r="G7"/>
     </row>
     <row r="8" spans="1:7" ht="15">
-      <c r="A8" s="73">
+      <c r="A8" s="70">
         <v>3</v>
       </c>
-      <c r="B8" s="71" t="s">
-        <v>311</v>
+      <c r="B8" s="69" t="s">
+        <v>330</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>312</v>
-      </c>
-      <c r="D8" s="69" t="s">
+        <v>331</v>
+      </c>
+      <c r="D8" s="76" t="s">
         <v>121</v>
       </c>
-      <c r="E8" s="67" t="s">
-        <v>313</v>
-      </c>
-      <c r="F8" s="67"/>
+      <c r="E8" s="74" t="s">
+        <v>332</v>
+      </c>
+      <c r="F8" s="74"/>
       <c r="G8"/>
     </row>
     <row r="9" spans="1:7" ht="30.75">
-      <c r="A9" s="73"/>
-      <c r="B9" s="71"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="69"/>
       <c r="C9" s="32" t="s">
-        <v>314</v>
-      </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="68"/>
-      <c r="F9" s="68"/>
+        <v>333</v>
+      </c>
+      <c r="D9" s="76"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
       <c r="G9"/>
     </row>
     <row r="10" spans="1:7" ht="15">
-      <c r="A10" s="72">
+      <c r="A10" s="73">
         <v>4</v>
       </c>
-      <c r="B10" s="75" t="s">
-        <v>315</v>
+      <c r="B10" s="72" t="s">
+        <v>334</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>316</v>
-      </c>
-      <c r="D10" s="72" t="s">
-        <v>317</v>
+        <v>335</v>
+      </c>
+      <c r="D10" s="73" t="s">
+        <v>336</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="F10" s="35"/>
       <c r="G10"/>
     </row>
     <row r="11" spans="1:7" ht="30.75">
-      <c r="A11" s="72"/>
-      <c r="B11" s="75"/>
+      <c r="A11" s="73"/>
+      <c r="B11" s="72"/>
       <c r="C11" s="36" t="s">
-        <v>319</v>
-      </c>
-      <c r="D11" s="72"/>
+        <v>338</v>
+      </c>
+      <c r="D11" s="73"/>
       <c r="E11" s="36" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="F11" s="36"/>
       <c r="G11"/>
     </row>
     <row r="12" spans="1:7" ht="15">
-      <c r="A12" s="72"/>
-      <c r="B12" s="75"/>
+      <c r="A12" s="73"/>
+      <c r="B12" s="72"/>
       <c r="C12" s="35" t="s">
-        <v>321</v>
-      </c>
-      <c r="D12" s="72"/>
+        <v>340</v>
+      </c>
+      <c r="D12" s="73"/>
       <c r="E12" s="35"/>
       <c r="F12" s="35"/>
       <c r="G12"/>
     </row>
     <row r="13" spans="1:7" ht="30.75">
-      <c r="A13" s="72"/>
-      <c r="B13" s="75"/>
+      <c r="A13" s="73"/>
+      <c r="B13" s="72"/>
       <c r="C13" s="36" t="s">
-        <v>307</v>
-      </c>
-      <c r="D13" s="72"/>
+        <v>326</v>
+      </c>
+      <c r="D13" s="73"/>
       <c r="E13" s="36"/>
       <c r="F13" s="36"/>
       <c r="G13"/>
     </row>
     <row r="14" spans="1:7" ht="15">
-      <c r="A14" s="73">
-        <v>5</v>
-      </c>
-      <c r="B14" s="71" t="s">
-        <v>322</v>
+      <c r="A14" s="70">
+        <v>5</v>
+      </c>
+      <c r="B14" s="69" t="s">
+        <v>341</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="D14" s="69" t="s">
+        <v>342</v>
+      </c>
+      <c r="D14" s="76" t="s">
         <v>145</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="F14" s="33"/>
       <c r="G14"/>
     </row>
     <row r="15" spans="1:7" ht="15">
-      <c r="A15" s="73"/>
-      <c r="B15" s="71"/>
+      <c r="A15" s="70"/>
+      <c r="B15" s="69"/>
       <c r="C15" s="32" t="s">
-        <v>325</v>
-      </c>
-      <c r="D15" s="69"/>
+        <v>344</v>
+      </c>
+      <c r="D15" s="76"/>
       <c r="E15" s="32" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="F15" s="32"/>
       <c r="G15"/>
     </row>
     <row r="16" spans="1:7" ht="30.75">
-      <c r="A16" s="73"/>
-      <c r="B16" s="71"/>
+      <c r="A16" s="70"/>
+      <c r="B16" s="69"/>
       <c r="C16" s="33" t="s">
-        <v>307</v>
-      </c>
-      <c r="D16" s="69"/>
+        <v>326</v>
+      </c>
+      <c r="D16" s="76"/>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
       <c r="G16"/>
@@ -7924,94 +8240,94 @@
         <v>6</v>
       </c>
       <c r="B17" s="36" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="D17" s="36"/>
       <c r="E17" s="36" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="F17" s="36"/>
       <c r="G17"/>
     </row>
     <row r="18" spans="1:7" ht="15">
-      <c r="A18" s="73">
+      <c r="A18" s="70">
         <v>7</v>
       </c>
-      <c r="B18" s="71" t="s">
-        <v>330</v>
+      <c r="B18" s="69" t="s">
+        <v>349</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>331</v>
-      </c>
-      <c r="D18" s="69" t="s">
+        <v>350</v>
+      </c>
+      <c r="D18" s="76" t="s">
         <v>144</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="F18" s="33"/>
       <c r="G18"/>
     </row>
     <row r="19" spans="1:7" ht="15">
-      <c r="A19" s="73"/>
-      <c r="B19" s="71"/>
+      <c r="A19" s="70"/>
+      <c r="B19" s="69"/>
       <c r="C19" s="32" t="s">
-        <v>332</v>
-      </c>
-      <c r="D19" s="69"/>
+        <v>351</v>
+      </c>
+      <c r="D19" s="76"/>
       <c r="E19" s="33" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="F19" s="32"/>
     </row>
     <row r="20" spans="1:7" ht="15">
-      <c r="A20" s="73"/>
-      <c r="B20" s="71"/>
+      <c r="A20" s="70"/>
+      <c r="B20" s="69"/>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
       <c r="E20" s="39"/>
       <c r="F20" s="37"/>
     </row>
     <row r="21" spans="1:7" ht="15">
-      <c r="A21" s="74">
+      <c r="A21" s="71">
         <v>8</v>
       </c>
-      <c r="B21" s="70" t="s">
-        <v>334</v>
+      <c r="B21" s="77" t="s">
+        <v>353</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="D21" s="40" t="s">
         <v>144</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="F21" s="40" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15">
-      <c r="A22" s="74"/>
-      <c r="B22" s="70"/>
+      <c r="A22" s="71"/>
+      <c r="B22" s="77"/>
       <c r="C22" s="35" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="D22" s="41" t="s">
         <v>70</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="F22" s="40"/>
     </row>
     <row r="23" spans="1:7" ht="15">
-      <c r="A23" s="74"/>
-      <c r="B23" s="70"/>
+      <c r="A23" s="71"/>
+      <c r="B23" s="77"/>
       <c r="C23" s="36"/>
       <c r="D23" s="36"/>
       <c r="E23" s="16"/>
@@ -8022,14 +8338,14 @@
         <v>9</v>
       </c>
       <c r="B24" s="32" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="D24" s="33"/>
       <c r="E24" s="33" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="F24" s="33"/>
     </row>
@@ -8140,13 +8456,14 @@
     <row r="86" ht="14.45" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="D8:D9"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="B18:B20"/>
@@ -8155,14 +8472,13 @@
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="A14:A16"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="D3:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8185,31 +8501,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="6" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15" customHeight="1">
@@ -8217,14 +8533,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="13" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="F2" s="14"/>
       <c r="G2" s="14"/>
@@ -8236,14 +8552,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="D3" s="12"/>
       <c r="E3" s="12" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="F3" s="14"/>
       <c r="G3" s="14"/>
@@ -8254,11 +8570,11 @@
       <c r="A4" s="11"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="12" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="F4" s="14"/>
       <c r="G4" s="14"/>
@@ -8269,7 +8585,7 @@
       <c r="A5" s="11"/>
       <c r="B5" s="12"/>
       <c r="C5" s="15" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="12"/>
@@ -8282,7 +8598,7 @@
       <c r="A6" s="11"/>
       <c r="B6" s="12"/>
       <c r="C6" s="12" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
@@ -8296,13 +8612,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
@@ -8315,13 +8631,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
@@ -8333,7 +8649,7 @@
       <c r="A9" s="11"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
@@ -8347,13 +8663,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
@@ -8365,10 +8681,10 @@
       <c r="A11" s="11"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
@@ -8380,7 +8696,7 @@
       <c r="A12" s="11"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="12"/>
@@ -8393,7 +8709,7 @@
       <c r="A13" s="11"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="12"/>
@@ -8407,13 +8723,13 @@
         <v>6</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
@@ -8425,10 +8741,10 @@
       <c r="A15" s="11"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
@@ -8440,7 +8756,7 @@
       <c r="A16" s="11"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
@@ -8454,13 +8770,13 @@
         <v>7</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
@@ -8473,13 +8789,13 @@
         <v>8</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
@@ -8491,10 +8807,10 @@
       <c r="A19" s="11"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="E19" s="12"/>
       <c r="F19" s="12"/>
@@ -8518,13 +8834,13 @@
         <v>9</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
@@ -8536,10 +8852,10 @@
       <c r="A22" s="11"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
@@ -8563,13 +8879,13 @@
         <v>10</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="E24" s="12"/>
       <c r="F24" s="12"/>
@@ -8582,12 +8898,12 @@
         <v>11</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="14"/>
@@ -8599,12 +8915,12 @@
         <v>12</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
       <c r="E26" s="12" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="14"/>

</xml_diff>